<commit_message>
fix data logs edit and logic login for users
</commit_message>
<xml_diff>
--- a/docs/test-cases/SDFish_TestCases_2026-07-02.xlsx
+++ b/docs/test-cases/SDFish_TestCases_2026-07-02.xlsx
@@ -7,6 +7,7 @@
     <sheet name="TA-010 Sắp xếp mức phạt" sheetId="3" r:id="rId3"/>
     <sheet name="BT-003 Hồ sơ chi tiết" sheetId="4" r:id="rId4"/>
     <sheet name="AUTH Ép đổi mật khẩu" sheetId="5" r:id="rId5"/>
+    <sheet name="SCOPE Data theo tài khoản" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -1689,4 +1690,323 @@
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE — Đăng xuất/đổi tài khoản phải xoá sạch data cũ (tàu, thuyền viên, sổ...)</t>
+        </is>
+      </c>
+      <c r="B1" s="0"/>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="H1" s="0"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã TC</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tên test case</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiền điều kiện</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bước thực hiện</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KQ thực tế</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trạng thái</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE-01</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng xuất xoá data tàu</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng nhập TK A, đã sửa tên tàu + mã tàu</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bấm Đăng xuất (chip tài khoản trang chủ) → xem chip tàu</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang tự tải lại; tàu về mặc định 'Tàu của tôi' — KHÔNG còn tên/mã tàu của A</t>
+        </is>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE-02</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng xuất xong KHÔNG sửa được tàu cũ</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vừa đăng xuất khỏi A</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bấm chip tàu → Sửa → đổi tên → Lưu → đăng nhập lại A</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa chỉ áp lên tàu mặc định mới; data tàu cũ của A KHÔNG quay lại (bug cũ: vẫn sửa được tàu của A)</t>
+        </is>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE-03</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đổi tài khoản A → B</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TK A có tàu + thuyền viên + sổ nợ</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng xuất A → đăng nhập B → xem /nguoi, /tien, chip tàu</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B thấy sổ TRỐNG/mặc định — không thấy bất kỳ data nào của A</t>
+        </is>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE-04</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thuyền viên + sổ nợ cũng bị xoá</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TK A có 2 thuyền viên, 1 chủ nợ</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng xuất → xem /nguoi và /tien tab Công nợ</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sổ thuyền viên về sổ mẫu/trống; công nợ trống</t>
+        </is>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE-05</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cài đặt giao diện được GIỮ</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã chọn 'Chữ to', lớp bản đồ vệ tinh</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng xuất</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cỡ chữ + lớp bản đồ + vùng nhà GIỮ nguyên (prefs theo máy, không theo tài khoản)</t>
+        </is>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE-06</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cùng tài khoản đăng nhập lại</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng nhập A, có data, KHÔNG đăng xuất</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tắt app mở lại / refresh trang</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data còn nguyên — không bị xoá oan, không reload lặp</t>
+        </is>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE-07</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đổi mật khẩu không mất data</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đang đăng nhập A có data</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đổi mật khẩu ở /doi-mat-khau</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data tàu/sổ giữ nguyên (cùng user — không reload, không xoá)</t>
+        </is>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE-08</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data không 'hồi sinh' sau đăng xuất</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TK A có tàu tên riêng</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng xuất → đợi trang tải lại xong → refresh thêm lần nữa</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tàu vẫn là mặc định — data A không quay lại sau bất kỳ refresh nào (race đã vá)</t>
+        </is>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ra-khoi): kho du lieu lich su + cron collector (0005)
</commit_message>
<xml_diff>
--- a/docs/test-cases/SDFish_TestCases_2026-07-02.xlsx
+++ b/docs/test-cases/SDFish_TestCases_2026-07-02.xlsx
@@ -7,8 +7,9 @@
     <sheet name="TA-010 Sắp xếp mức phạt" sheetId="3" r:id="rId3"/>
     <sheet name="BT-003 Hồ sơ chi tiết" sheetId="4" r:id="rId4"/>
     <sheet name="AUTH Ép đổi mật khẩu" sheetId="5" r:id="rId5"/>
-    <sheet name="DMK Đổi mật khẩu" sheetId="6" r:id="rId6"/>
-    <sheet name="SCOPE Data theo tài khoản" sheetId="7" r:id="rId7"/>
+    <sheet name="RKDB Lưu lịch sử Ra khơi" sheetId="6" r:id="rId6"/>
+    <sheet name="DMK Đổi mật khẩu" sheetId="7" r:id="rId7"/>
+    <sheet name="SCOPE Data theo tài khoản" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -1711,7 +1712,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK — Nút Đổi mật khẩu trong sheet Tài khoản (mở khoá DN-001-04/07)</t>
+          <t xml:space="preserve">RKDB — Cron lưu dữ liệu Ra khơi vào DB (predict) — test kỹ thuật, cần secret</t>
         </is>
       </c>
       <c r="B1" s="0"/>
@@ -1767,27 +1768,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-01</t>
+          <t xml:space="preserve">RKDB-01</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thấy nút khi đã đăng nhập</t>
+          <t xml:space="preserve">Chặn người lạ</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã đăng nhập</t>
+          <t xml:space="preserve">Đã deploy, có CRON_SECRET</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang chủ → bấm chip tài khoản (tên/SĐT) → xem sheet</t>
+          <t xml:space="preserve">GET /api/collect/sea-daily KHÔNG kèm Authorization</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Có nút 'Đổi mật khẩu' phía trên nút Đăng xuất</t>
+          <t xml:space="preserve">401 unauthorized</t>
         </is>
       </c>
       <c r="F3" s="3"/>
@@ -1797,27 +1798,27 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-02</t>
+          <t xml:space="preserve">RKDB-02</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ẩn nút khi chưa đăng nhập</t>
+          <t xml:space="preserve">Sai secret</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chưa đăng nhập</t>
+          <t xml:space="preserve">Như trên</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang chủ → bấm chip 'Đăng nhập' → xem sheet</t>
+          <t xml:space="preserve">GET kèm 'Authorization: Bearer sai'</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">KHÔNG có nút Đổi mật khẩu — chỉ thấy nút Đăng nhập / Đăng ký</t>
+          <t xml:space="preserve">401 unauthorized</t>
         </is>
       </c>
       <c r="F4" s="3"/>
@@ -1827,27 +1828,27 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-03</t>
+          <t xml:space="preserve">RKDB-03</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nút mở đúng trang</t>
+          <t xml:space="preserve">Chạy tay đúng secret</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã đăng nhập</t>
+          <t xml:space="preserve">Migration 0005 đã apply</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bấm 'Đổi mật khẩu' trong sheet</t>
+          <t xml:space="preserve">GET kèm Bearer đúng CRON_SECRET</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sheet đóng, mở trang /doi-mat-khau với form 2 ô mật khẩu</t>
+          <t xml:space="preserve">200; parts.sea.ok=true, rows=100 (10 cảng × 10 ngày)</t>
         </is>
       </c>
       <c r="F5" s="3"/>
@@ -1857,27 +1858,27 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-04</t>
+          <t xml:space="preserve">RKDB-04</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đổi mật khẩu thành công</t>
+          <t xml:space="preserve">Dữ liệu sea_daily đúng</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đang ở trang đổi MK</t>
+          <t xml:space="preserve">Vừa chạy RKDB-03</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhập MK mới hợp lệ 2 ô khớp nhau → Lưu</t>
+          <t xml:space="preserve">Query Supabase: select * from sea_daily where collected_on = hôm nay</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Về trang chính; đăng xuất → đăng nhập lại bằng MK MỚI vào được, MK CŨ báo sai</t>
+          <t xml:space="preserve">100 hàng; lead_days 0–9; score 1–100; wave/wind/mưa có số</t>
         </is>
       </c>
       <c r="F6" s="3"/>
@@ -1887,27 +1888,27 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-05</t>
+          <t xml:space="preserve">RKDB-05</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 ô không khớp</t>
+          <t xml:space="preserve">Hotspot cá được lưu</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang đổi MK</t>
+          <t xml:space="preserve">NOAA hoạt động (chạy trên Vercel)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ô 1 ≠ ô 2 → Lưu</t>
+          <t xml:space="preserve">Query fish_forecast_daily theo collected_on</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo 'Hai ô mật khẩu chưa giống nhau', không lưu</t>
+          <t xml:space="preserve">Các hàng score ≥ 60, có loài + toạ độ + SST</t>
         </is>
       </c>
       <c r="F7" s="3"/>
@@ -1917,27 +1918,27 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-06</t>
+          <t xml:space="preserve">RKDB-06</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MK quá ngắn</t>
+          <t xml:space="preserve">Chạy lại trong ngày không nhân đôi</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang đổi MK</t>
+          <t xml:space="preserve">Vừa chạy RKDB-03</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhập MK 5 ký tự → Lưu</t>
+          <t xml:space="preserve">Gọi lại route lần 2 cùng ngày → đếm lại hàng</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo 'ít nhất 6 ký tự', không lưu</t>
+          <t xml:space="preserve">Số hàng KHÔNG đổi (upsert idempotent)</t>
         </is>
       </c>
       <c r="F8" s="3"/>
@@ -1947,27 +1948,27 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-07</t>
+          <t xml:space="preserve">RKDB-07</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vào URL khi chưa đăng nhập</t>
+          <t xml:space="preserve">Cron tự chạy</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chưa đăng nhập</t>
+          <t xml:space="preserve">Deploy qua đêm</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gõ thẳng /doi-mat-khau</t>
+          <t xml:space="preserve">Sáng hôm sau (sau 6:30 VN) query collected_on = hôm nay</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hiện lời mời đăng nhập + nút Đăng nhập — KHÔNG hiện form đổi</t>
+          <t xml:space="preserve">Có data mới tự động, không ai bấm gì</t>
         </is>
       </c>
       <c r="F9" s="3"/>
@@ -1977,27 +1978,27 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-08</t>
+          <t xml:space="preserve">RKDB-08</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chạy lại DN-001-04 + DN-001-07</t>
+          <t xml:space="preserve">Client không đọc được bảng</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đổi MK được rồi</t>
+          <t xml:space="preserve">Đăng nhập app bằng acc thường</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đặt MK có khoảng trắng đầu/cuối và MK cụm từ có khoảng trắng giữa theo 2 case sheet DN-001</t>
+          <t xml:space="preserve">Dùng anon key query sea_daily</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DN-001-04: vào được bằng đúng cụm từ; DN-001-07: đăng nhập được bằng bản không dư khoảng trắng</t>
+          <t xml:space="preserve">0 hàng / từ chối (RLS đóng — chỉ service-role)</t>
         </is>
       </c>
       <c r="F10" s="3"/>
@@ -2030,7 +2031,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SCOPE — Đăng xuất/đổi tài khoản phải xoá sạch data cũ (tàu, thuyền viên, sổ...)</t>
+          <t xml:space="preserve">DMK — Nút Đổi mật khẩu trong sheet Tài khoản (mở khoá DN-001-04/07)</t>
         </is>
       </c>
       <c r="B1" s="0"/>
@@ -2086,6 +2087,325 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">DMK-01</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thấy nút khi đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang chủ → bấm chip tài khoản (tên/SĐT) → xem sheet</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có nút 'Đổi mật khẩu' phía trên nút Đăng xuất</t>
+        </is>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-02</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ẩn nút khi chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang chủ → bấm chip 'Đăng nhập' → xem sheet</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KHÔNG có nút Đổi mật khẩu — chỉ thấy nút Đăng nhập / Đăng ký</t>
+        </is>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-03</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nút mở đúng trang</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bấm 'Đổi mật khẩu' trong sheet</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sheet đóng, mở trang /doi-mat-khau với form 2 ô mật khẩu</t>
+        </is>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-04</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đổi mật khẩu thành công</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đang ở trang đổi MK</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nhập MK mới hợp lệ 2 ô khớp nhau → Lưu</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Về trang chính; đăng xuất → đăng nhập lại bằng MK MỚI vào được, MK CŨ báo sai</t>
+        </is>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-05</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 ô không khớp</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang đổi MK</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ô 1 ≠ ô 2 → Lưu</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Báo 'Hai ô mật khẩu chưa giống nhau', không lưu</t>
+        </is>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-06</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MK quá ngắn</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang đổi MK</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nhập MK 5 ký tự → Lưu</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Báo 'ít nhất 6 ký tự', không lưu</t>
+        </is>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-07</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vào URL khi chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gõ thẳng /doi-mat-khau</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hiện lời mời đăng nhập + nút Đăng nhập — KHÔNG hiện form đổi</t>
+        </is>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-08</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chạy lại DN-001-04 + DN-001-07</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đổi MK được rồi</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đặt MK có khoảng trắng đầu/cuối và MK cụm từ có khoảng trắng giữa theo 2 case sheet DN-001</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DN-001-04: vào được bằng đúng cụm từ; DN-001-07: đăng nhập được bằng bản không dư khoảng trắng</t>
+        </is>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE — Đăng xuất/đổi tài khoản phải xoá sạch data cũ (tàu, thuyền viên, sổ...)</t>
+        </is>
+      </c>
+      <c r="B1" s="0"/>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="H1" s="0"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã TC</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tên test case</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiền điều kiện</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bước thực hiện</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KQ thực tế</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trạng thái</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">SCOPE-01</t>
         </is>
       </c>

</xml_diff>

<commit_message>
fix logic create login accounts, rls, trigger
</commit_message>
<xml_diff>
--- a/docs/test-cases/SDFish_TestCases_2026-07-02.xlsx
+++ b/docs/test-cases/SDFish_TestCases_2026-07-02.xlsx
@@ -7,9 +7,10 @@
     <sheet name="TA-010 Sắp xếp mức phạt" sheetId="3" r:id="rId3"/>
     <sheet name="BT-003 Hồ sơ chi tiết" sheetId="4" r:id="rId4"/>
     <sheet name="AUTH Ép đổi mật khẩu" sheetId="5" r:id="rId5"/>
-    <sheet name="RKDB Lưu lịch sử Ra khơi" sheetId="6" r:id="rId6"/>
-    <sheet name="DMK Đổi mật khẩu" sheetId="7" r:id="rId7"/>
-    <sheet name="SCOPE Data theo tài khoản" sheetId="8" r:id="rId8"/>
+    <sheet name="RK002 Dự báo cá" sheetId="6" r:id="rId6"/>
+    <sheet name="RKDB Lưu lịch sử Ra khơi" sheetId="7" r:id="rId7"/>
+    <sheet name="DMK Đổi mật khẩu" sheetId="8" r:id="rId8"/>
+    <sheet name="SCOPE Data theo tài khoản" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -1696,7 +1697,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1712,7 +1713,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RKDB — Cron lưu dữ liệu Ra khơi vào DB (predict) — test kỹ thuật, cần secret</t>
+          <t xml:space="preserve">RK-002 — Lớp dự báo cá tải được (fix 403 nguồn NOAA, 07/07)</t>
         </is>
       </c>
       <c r="B1" s="0"/>
@@ -1768,27 +1769,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RKDB-01</t>
+          <t xml:space="preserve">RK002-01</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chặn người lạ</t>
+          <t xml:space="preserve">Lớp cá hiện trên bản đồ</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã deploy, có CRON_SECRET</t>
+          <t xml:space="preserve">Mở app trên mạng bình thường</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GET /api/collect/sea-daily KHÔNG kèm Authorization</t>
+          <t xml:space="preserve">Vào Ra khơi → chờ bản đồ → bật lớp Dự báo cá</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">401 unauthorized</t>
+          <t xml:space="preserve">Heatmap + điểm nóng cá hiển thị (không còn 'Dự báo cá chưa tải được')</t>
         </is>
       </c>
       <c r="F3" s="3"/>
@@ -1798,27 +1799,27 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RKDB-02</t>
+          <t xml:space="preserve">RK002-02</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sai secret</t>
+          <t xml:space="preserve">Chạm điểm nóng khi CHƯA đăng nhập</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Như trên</t>
+          <t xml:space="preserve">Chưa đăng nhập</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GET kèm 'Authorization: Bearer sai'</t>
+          <t xml:space="preserve">Chạm 1 điểm nóng cá</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">401 unauthorized</t>
+          <t xml:space="preserve">Thấy mời đăng nhập để xem chi tiết (teaser đúng thiết kế)</t>
         </is>
       </c>
       <c r="F4" s="3"/>
@@ -1828,27 +1829,27 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RKDB-03</t>
+          <t xml:space="preserve">RK002-03</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chạy tay đúng secret</t>
+          <t xml:space="preserve">Chạm điểm nóng khi ĐÃ đăng nhập</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Migration 0005 đã apply</t>
+          <t xml:space="preserve">Đã đăng nhập</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GET kèm Bearer đúng CRON_SECRET</t>
+          <t xml:space="preserve">Chạm 1 điểm nóng cá</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">200; parts.sea.ok=true, rows=100 (10 cảng × 10 ngày)</t>
+          <t xml:space="preserve">Hiện chi tiết: loài, khả năng, nhiệt độ nước, phù du</t>
         </is>
       </c>
       <c r="F5" s="3"/>
@@ -1858,27 +1859,27 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RKDB-04</t>
+          <t xml:space="preserve">RK002-04</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dữ liệu sea_daily đúng</t>
+          <t xml:space="preserve">Ngày ảnh nguồn trung thực</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vừa chạy RKDB-03</t>
+          <t xml:space="preserve">Lớp cá đang hiện</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Query Supabase: select * from sea_daily where collected_on = hôm nay</t>
+          <t xml:space="preserve">Xem nhãn ngày cập nhật của lớp cá</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">100 hàng; lead_days 0–9; score 1–100; wave/wind/mưa có số</t>
+          <t xml:space="preserve">Ghi rõ ngày ảnh vệ tinh (có thể trễ 1-2 ngày — đúng, không bịa)</t>
         </is>
       </c>
       <c r="F6" s="3"/>
@@ -1888,122 +1889,32 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RKDB-05</t>
+          <t xml:space="preserve">RK002-05</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hotspot cá được lưu</t>
+          <t xml:space="preserve">Hotspot được lưu vào kho</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">NOAA hoạt động (chạy trên Vercel)</t>
+          <t xml:space="preserve">Sau 6:30 sáng (cron đã chạy)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Query fish_forecast_daily theo collected_on</t>
+          <t xml:space="preserve">Query fish_forecast_daily theo collected_on hôm nay</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Các hàng score ≥ 60, có loài + toạ độ + SST</t>
+          <t xml:space="preserve">Có hàng hotspot (score ≥ 60) kèm loài + SST</t>
         </is>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RKDB-06</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chạy lại trong ngày không nhân đôi</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vừa chạy RKDB-03</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gọi lại route lần 2 cùng ngày → đếm lại hàng</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số hàng KHÔNG đổi (upsert idempotent)</t>
-        </is>
-      </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RKDB-07</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cron tự chạy</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Deploy qua đêm</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sáng hôm sau (sau 6:30 VN) query collected_on = hôm nay</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có data mới tự động, không ai bấm gì</t>
-        </is>
-      </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RKDB-08</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Client không đọc được bảng</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đăng nhập app bằng acc thường</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dùng anon key query sea_daily</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0 hàng / từ chối (RLS đóng — chỉ service-role)</t>
-        </is>
-      </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2031,7 +1942,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK — Nút Đổi mật khẩu trong sheet Tài khoản (mở khoá DN-001-04/07)</t>
+          <t xml:space="preserve">RKDB — Cron lưu dữ liệu Ra khơi vào DB (predict) — test kỹ thuật, cần secret</t>
         </is>
       </c>
       <c r="B1" s="0"/>
@@ -2087,27 +1998,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-01</t>
+          <t xml:space="preserve">RKDB-01</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thấy nút khi đã đăng nhập</t>
+          <t xml:space="preserve">Chặn người lạ</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã đăng nhập</t>
+          <t xml:space="preserve">Đã deploy, có CRON_SECRET</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang chủ → bấm chip tài khoản (tên/SĐT) → xem sheet</t>
+          <t xml:space="preserve">GET /api/collect/sea-daily KHÔNG kèm Authorization</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Có nút 'Đổi mật khẩu' phía trên nút Đăng xuất</t>
+          <t xml:space="preserve">401 unauthorized</t>
         </is>
       </c>
       <c r="F3" s="3"/>
@@ -2117,27 +2028,27 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-02</t>
+          <t xml:space="preserve">RKDB-02</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ẩn nút khi chưa đăng nhập</t>
+          <t xml:space="preserve">Sai secret</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chưa đăng nhập</t>
+          <t xml:space="preserve">Như trên</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang chủ → bấm chip 'Đăng nhập' → xem sheet</t>
+          <t xml:space="preserve">GET kèm 'Authorization: Bearer sai'</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">KHÔNG có nút Đổi mật khẩu — chỉ thấy nút Đăng nhập / Đăng ký</t>
+          <t xml:space="preserve">401 unauthorized</t>
         </is>
       </c>
       <c r="F4" s="3"/>
@@ -2147,27 +2058,27 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-03</t>
+          <t xml:space="preserve">RKDB-03</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nút mở đúng trang</t>
+          <t xml:space="preserve">Chạy tay đúng secret</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã đăng nhập</t>
+          <t xml:space="preserve">Migration 0005 đã apply</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bấm 'Đổi mật khẩu' trong sheet</t>
+          <t xml:space="preserve">GET kèm Bearer đúng CRON_SECRET</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sheet đóng, mở trang /doi-mat-khau với form 2 ô mật khẩu</t>
+          <t xml:space="preserve">200; parts.sea.ok=true, rows=100 (10 cảng × 10 ngày)</t>
         </is>
       </c>
       <c r="F5" s="3"/>
@@ -2177,27 +2088,27 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-04</t>
+          <t xml:space="preserve">RKDB-04</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đổi mật khẩu thành công</t>
+          <t xml:space="preserve">Dữ liệu sea_daily đúng</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đang ở trang đổi MK</t>
+          <t xml:space="preserve">Vừa chạy RKDB-03</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhập MK mới hợp lệ 2 ô khớp nhau → Lưu</t>
+          <t xml:space="preserve">Query Supabase: select * from sea_daily where collected_on = hôm nay</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Về trang chính; đăng xuất → đăng nhập lại bằng MK MỚI vào được, MK CŨ báo sai</t>
+          <t xml:space="preserve">100 hàng; lead_days 0–9; score 1–100; wave/wind/mưa có số</t>
         </is>
       </c>
       <c r="F6" s="3"/>
@@ -2207,27 +2118,27 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-05</t>
+          <t xml:space="preserve">RKDB-05</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 ô không khớp</t>
+          <t xml:space="preserve">Hotspot cá được lưu</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang đổi MK</t>
+          <t xml:space="preserve">NOAA hoạt động (chạy trên Vercel)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ô 1 ≠ ô 2 → Lưu</t>
+          <t xml:space="preserve">Query fish_forecast_daily theo collected_on</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo 'Hai ô mật khẩu chưa giống nhau', không lưu</t>
+          <t xml:space="preserve">Các hàng score ≥ 60, có loài + toạ độ + SST</t>
         </is>
       </c>
       <c r="F7" s="3"/>
@@ -2237,27 +2148,27 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-06</t>
+          <t xml:space="preserve">RKDB-06</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MK quá ngắn</t>
+          <t xml:space="preserve">Chạy lại trong ngày không nhân đôi</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang đổi MK</t>
+          <t xml:space="preserve">Vừa chạy RKDB-03</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhập MK 5 ký tự → Lưu</t>
+          <t xml:space="preserve">Gọi lại route lần 2 cùng ngày → đếm lại hàng</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo 'ít nhất 6 ký tự', không lưu</t>
+          <t xml:space="preserve">Số hàng KHÔNG đổi (upsert idempotent)</t>
         </is>
       </c>
       <c r="F8" s="3"/>
@@ -2267,27 +2178,27 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-07</t>
+          <t xml:space="preserve">RKDB-07</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vào URL khi chưa đăng nhập</t>
+          <t xml:space="preserve">Cron tự chạy</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chưa đăng nhập</t>
+          <t xml:space="preserve">Deploy qua đêm</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gõ thẳng /doi-mat-khau</t>
+          <t xml:space="preserve">Sáng hôm sau (sau 6:30 VN) query collected_on = hôm nay</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hiện lời mời đăng nhập + nút Đăng nhập — KHÔNG hiện form đổi</t>
+          <t xml:space="preserve">Có data mới tự động, không ai bấm gì</t>
         </is>
       </c>
       <c r="F9" s="3"/>
@@ -2297,27 +2208,27 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMK-08</t>
+          <t xml:space="preserve">RKDB-08</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chạy lại DN-001-04 + DN-001-07</t>
+          <t xml:space="preserve">Client không đọc được bảng</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đổi MK được rồi</t>
+          <t xml:space="preserve">Đăng nhập app bằng acc thường</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đặt MK có khoảng trắng đầu/cuối và MK cụm từ có khoảng trắng giữa theo 2 case sheet DN-001</t>
+          <t xml:space="preserve">Dùng anon key query sea_daily</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DN-001-04: vào được bằng đúng cụm từ; DN-001-07: đăng nhập được bằng bản không dư khoảng trắng</t>
+          <t xml:space="preserve">0 hàng / từ chối (RLS đóng — chỉ service-role)</t>
         </is>
       </c>
       <c r="F10" s="3"/>
@@ -2350,7 +2261,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SCOPE — Đăng xuất/đổi tài khoản phải xoá sạch data cũ (tàu, thuyền viên, sổ...)</t>
+          <t xml:space="preserve">DMK — Nút Đổi mật khẩu trong sheet Tài khoản (mở khoá DN-001-04/07)</t>
         </is>
       </c>
       <c r="B1" s="0"/>
@@ -2406,6 +2317,325 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">DMK-01</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thấy nút khi đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang chủ → bấm chip tài khoản (tên/SĐT) → xem sheet</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có nút 'Đổi mật khẩu' phía trên nút Đăng xuất</t>
+        </is>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-02</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ẩn nút khi chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang chủ → bấm chip 'Đăng nhập' → xem sheet</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KHÔNG có nút Đổi mật khẩu — chỉ thấy nút Đăng nhập / Đăng ký</t>
+        </is>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-03</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nút mở đúng trang</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bấm 'Đổi mật khẩu' trong sheet</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sheet đóng, mở trang /doi-mat-khau với form 2 ô mật khẩu</t>
+        </is>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-04</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đổi mật khẩu thành công</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đang ở trang đổi MK</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nhập MK mới hợp lệ 2 ô khớp nhau → Lưu</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Về trang chính; đăng xuất → đăng nhập lại bằng MK MỚI vào được, MK CŨ báo sai</t>
+        </is>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-05</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 ô không khớp</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang đổi MK</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ô 1 ≠ ô 2 → Lưu</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Báo 'Hai ô mật khẩu chưa giống nhau', không lưu</t>
+        </is>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-06</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MK quá ngắn</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang đổi MK</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nhập MK 5 ký tự → Lưu</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Báo 'ít nhất 6 ký tự', không lưu</t>
+        </is>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-07</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vào URL khi chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gõ thẳng /doi-mat-khau</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hiện lời mời đăng nhập + nút Đăng nhập — KHÔNG hiện form đổi</t>
+        </is>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DMK-08</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chạy lại DN-001-04 + DN-001-07</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đổi MK được rồi</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đặt MK có khoảng trắng đầu/cuối và MK cụm từ có khoảng trắng giữa theo 2 case sheet DN-001</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DN-001-04: vào được bằng đúng cụm từ; DN-001-07: đăng nhập được bằng bản không dư khoảng trắng</t>
+        </is>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCOPE — Đăng xuất/đổi tài khoản phải xoá sạch data cũ (tàu, thuyền viên, sổ...)</t>
+        </is>
+      </c>
+      <c r="B1" s="0"/>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="H1" s="0"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã TC</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tên test case</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiền điều kiện</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bước thực hiện</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KQ thực tế</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trạng thái</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">SCOPE-01</t>
         </is>
       </c>

</xml_diff>